<commit_message>
fix: chart below Tribe Scorecard Summary, 60x44cm doubled size, squad names on axis
</commit_message>
<xml_diff>
--- a/snapshots/2026-06-25/maturity-export-2026-06-25-report.xlsx
+++ b/snapshots/2026-06-25/maturity-export-2026-06-25-report.xlsx
@@ -302,9 +302,29 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <strRef>
-              <f>'Tribe Overview'!W3</f>
-            </strRef>
+            <v>Entities</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tribe Overview'!$A$4:$A$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tribe Overview'!$B$4:$B$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Rows</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -319,30 +339,6 @@
           <val>
             <numRef>
               <f>'Tribe Overview'!$W$4:$W$20</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Tribe Overview'!V3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Tribe Overview'!$A$4:$A$20</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Tribe Overview'!$V$4:$V$20</f>
             </numRef>
           </val>
         </ser>
@@ -388,10 +384,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="21600000" cy="15840000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>

</xml_diff>

<commit_message>
fix: chart shows squad names — add delete/tickLblPos to catAx, match 2026-06-20 size exactly
</commit_message>
<xml_diff>
--- a/snapshots/2026-06-25/maturity-export-2026-06-25-report.xlsx
+++ b/snapshots/2026-06-25/maturity-export-2026-06-25-report.xlsx
@@ -302,7 +302,9 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>Entities</v>
+            <strRef>
+              <f>'Tribe Overview'!B3</f>
+            </strRef>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -310,9 +312,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Tribe Overview'!$A$4:$A$20</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -324,7 +326,9 @@
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <v>Rows</v>
+            <strRef>
+              <f>'Tribe Overview'!W3</f>
+            </strRef>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -332,9 +336,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Tribe Overview'!$A$4:$A$20</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -351,9 +355,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -362,7 +368,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -387,7 +393,7 @@
       <row>34</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="21600000" cy="15840000"/>
+    <ext cx="10800000" cy="7920000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>

</xml_diff>